<commit_message>
Create combined data table
</commit_message>
<xml_diff>
--- a/Data/National-Imaging-Data-Collection-Asset-Count-2023-24-v1.xlsx
+++ b/Data/National-Imaging-Data-Collection-Asset-Count-2023-24-v1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\O46BTKGR\OneDrive - NHS\OI Diagnostics\15 Imaging\02 NIDC\03 NIDC Publication\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://healthsharedservice-my.sharepoint.com/personal/anne_foulger_dhsc_gov_uk/Documents/repos/FLS_mapping/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EC4695B-F8E4-41FF-BD0D-34AFA54B2EE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{0EC4695B-F8E4-41FF-BD0D-34AFA54B2EE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{18278FB5-C788-40E6-B090-3062EE4C846A}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{79F2D076-C940-4B30-8FDD-1AECEE309C4D}"/>
+    <workbookView xWindow="240" yWindow="0" windowWidth="8660" windowHeight="10060" activeTab="2" xr2:uid="{79F2D076-C940-4B30-8FDD-1AECEE309C4D}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="21" r:id="rId1"/>
@@ -20,7 +20,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ICB, Imaging Network and Trust'!$B$14:$S$152</definedName>
   </definedNames>
-  <calcPr calcId="191028" concurrentCalc="0"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -2180,19 +2180,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA835F15-C7B1-49E4-B38C-5A7B4039B0E7}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="B2:G33"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="2.140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="28.85546875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="33.5703125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="59.85546875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="2.1796875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="28.81640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="33.54296875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="59.81640625" style="1" customWidth="1"/>
     <col min="5" max="5" width="42" style="1" customWidth="1"/>
-    <col min="6" max="12" width="6.85546875" style="1" customWidth="1"/>
-    <col min="13" max="16384" width="9.140625" style="1"/>
+    <col min="6" max="12" width="6.81640625" style="1" customWidth="1"/>
+    <col min="13" max="16384" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="2:7" ht="35.25" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:7" ht="6" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="3" spans="2:7" ht="35" x14ac:dyDescent="0.35">
       <c r="B3" s="60" t="s">
         <v>400</v>
       </c>
@@ -2200,7 +2200,7 @@
       <c r="D3" s="61"/>
       <c r="E3" s="61"/>
     </row>
-    <row r="5" spans="2:7" ht="18" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:7" ht="18" x14ac:dyDescent="0.4">
       <c r="B5" s="2" t="s">
         <v>1</v>
       </c>
@@ -2208,7 +2208,7 @@
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
     </row>
-    <row r="6" spans="2:7" ht="95.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:7" ht="95.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="62" t="s">
         <v>2</v>
       </c>
@@ -2217,7 +2217,7 @@
       <c r="E6" s="63"/>
       <c r="G6" s="5"/>
     </row>
-    <row r="7" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B7" s="2" t="s">
         <v>3</v>
       </c>
@@ -2225,7 +2225,7 @@
       <c r="D7" s="4"/>
       <c r="E7" s="4"/>
     </row>
-    <row r="8" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B8" s="8" t="s">
         <v>4</v>
       </c>
@@ -2233,7 +2233,7 @@
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
     </row>
-    <row r="9" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B9" s="8" t="s">
         <v>5</v>
       </c>
@@ -2241,7 +2241,7 @@
       <c r="D9" s="4"/>
       <c r="E9" s="4"/>
     </row>
-    <row r="10" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B10" s="8" t="s">
         <v>6</v>
       </c>
@@ -2249,20 +2249,20 @@
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
     </row>
-    <row r="11" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B11" s="6"/>
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
       <c r="E11" s="4"/>
     </row>
-    <row r="12" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C12" s="12" t="s">
         <v>7</v>
       </c>
       <c r="D12" s="4"/>
       <c r="E12" s="4"/>
     </row>
-    <row r="13" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B13" s="7" t="s">
         <v>8</v>
       </c>
@@ -2272,7 +2272,7 @@
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
     </row>
-    <row r="14" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B14" s="7" t="s">
         <v>9</v>
       </c>
@@ -2282,7 +2282,7 @@
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
     </row>
-    <row r="15" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B15" s="57" t="s">
         <v>10</v>
       </c>
@@ -2292,7 +2292,7 @@
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
     </row>
-    <row r="16" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B16" s="59"/>
       <c r="C16" s="9" t="s">
         <v>12</v>
@@ -2300,7 +2300,7 @@
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
     </row>
-    <row r="17" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B17" s="59"/>
       <c r="C17" s="9" t="s">
         <v>13</v>
@@ -2308,7 +2308,7 @@
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
     </row>
-    <row r="18" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B18" s="58"/>
       <c r="C18" s="9" t="s">
         <v>14</v>
@@ -2316,7 +2316,7 @@
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
     </row>
-    <row r="19" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B19" s="57" t="s">
         <v>15</v>
       </c>
@@ -2326,7 +2326,7 @@
       <c r="D19" s="4"/>
       <c r="E19" s="4"/>
     </row>
-    <row r="20" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B20" s="58"/>
       <c r="C20" s="9" t="s">
         <v>17</v>
@@ -2334,7 +2334,7 @@
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
     </row>
-    <row r="21" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B21" s="7" t="s">
         <v>18</v>
       </c>
@@ -2344,7 +2344,7 @@
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
     </row>
-    <row r="22" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B22" s="7" t="s">
         <v>19</v>
       </c>
@@ -2354,7 +2354,7 @@
       <c r="D22" s="4"/>
       <c r="E22" s="4"/>
     </row>
-    <row r="23" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B23" s="64" t="s">
         <v>20</v>
       </c>
@@ -2364,7 +2364,7 @@
       <c r="D23" s="4"/>
       <c r="E23" s="4"/>
     </row>
-    <row r="24" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B24" s="65"/>
       <c r="C24" s="9" t="s">
         <v>21</v>
@@ -2372,7 +2372,7 @@
       <c r="D24" s="4"/>
       <c r="E24" s="4"/>
     </row>
-    <row r="25" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B25" s="7" t="s">
         <v>22</v>
       </c>
@@ -2382,7 +2382,7 @@
       <c r="D25" s="4"/>
       <c r="E25" s="4"/>
     </row>
-    <row r="26" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B26" s="7" t="s">
         <v>23</v>
       </c>
@@ -2392,7 +2392,7 @@
       <c r="D26" s="4"/>
       <c r="E26" s="4"/>
     </row>
-    <row r="27" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B27" s="7" t="s">
         <v>24</v>
       </c>
@@ -2402,7 +2402,7 @@
       <c r="D27" s="4"/>
       <c r="E27" s="4"/>
     </row>
-    <row r="28" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B28" s="7" t="s">
         <v>25</v>
       </c>
@@ -2412,13 +2412,13 @@
       <c r="D28" s="4"/>
       <c r="E28" s="4"/>
     </row>
-    <row r="29" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B29" s="6"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
       <c r="E29" s="4"/>
     </row>
-    <row r="30" spans="2:5" ht="18" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:5" ht="18" x14ac:dyDescent="0.4">
       <c r="B30" s="2" t="s">
         <v>26</v>
       </c>
@@ -2426,20 +2426,20 @@
       <c r="D30" s="4"/>
       <c r="E30" s="4"/>
     </row>
-    <row r="31" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B31" s="4" t="s">
         <v>27</v>
       </c>
       <c r="C31" s="4"/>
       <c r="D31" s="4"/>
     </row>
-    <row r="32" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
       <c r="D32" s="4"/>
       <c r="E32" s="4"/>
     </row>
-    <row r="33" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B33" s="11" t="s">
         <v>28</v>
       </c>
@@ -2464,19 +2464,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F612F52-003C-4311-BB27-405317FCBADD}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:T27"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="2.42578125" style="4" customWidth="1"/>
-    <col min="2" max="2" width="13.42578125" style="4" customWidth="1"/>
-    <col min="3" max="3" width="27.5703125" style="4" customWidth="1"/>
-    <col min="4" max="6" width="16.7109375" style="4" customWidth="1"/>
-    <col min="7" max="15" width="16.7109375" style="16" customWidth="1"/>
-    <col min="16" max="18" width="21.28515625" style="16" customWidth="1"/>
-    <col min="19" max="20" width="9.140625" style="16"/>
-    <col min="21" max="16384" width="9.140625" style="4"/>
+    <col min="1" max="1" width="2.453125" style="4" customWidth="1"/>
+    <col min="2" max="2" width="13.453125" style="4" customWidth="1"/>
+    <col min="3" max="3" width="27.54296875" style="4" customWidth="1"/>
+    <col min="4" max="6" width="16.7265625" style="4" customWidth="1"/>
+    <col min="7" max="15" width="16.7265625" style="16" customWidth="1"/>
+    <col min="16" max="18" width="21.26953125" style="16" customWidth="1"/>
+    <col min="19" max="20" width="9.1796875" style="16"/>
+    <col min="21" max="16384" width="9.1796875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="69"/>
       <c r="B1" s="69"/>
       <c r="C1" s="14"/>
@@ -2486,7 +2486,7 @@
       <c r="G1" s="15"/>
       <c r="H1" s="15"/>
     </row>
-    <row r="2" spans="1:18" ht="18" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:18" ht="18" x14ac:dyDescent="0.35">
       <c r="A2" s="13"/>
       <c r="B2" s="17" t="s">
         <v>29</v>
@@ -2500,7 +2500,7 @@
       <c r="G2" s="15"/>
       <c r="H2" s="15"/>
     </row>
-    <row r="3" spans="1:18" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A3" s="13"/>
       <c r="B3" s="17" t="s">
         <v>30</v>
@@ -2514,7 +2514,7 @@
       <c r="G3" s="15"/>
       <c r="H3" s="15"/>
     </row>
-    <row r="4" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A4" s="13"/>
       <c r="B4" s="19" t="s">
         <v>31</v>
@@ -2528,7 +2528,7 @@
       <c r="G4" s="15"/>
       <c r="H4" s="15"/>
     </row>
-    <row r="5" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A5" s="13"/>
       <c r="B5" s="19" t="s">
         <v>33</v>
@@ -2542,7 +2542,7 @@
       <c r="G5" s="15"/>
       <c r="H5" s="15"/>
     </row>
-    <row r="6" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A6" s="13"/>
       <c r="B6" s="19" t="s">
         <v>34</v>
@@ -2556,7 +2556,7 @@
       <c r="G6" s="15"/>
       <c r="H6" s="15"/>
     </row>
-    <row r="7" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A7" s="13"/>
       <c r="B7" s="19" t="s">
         <v>36</v>
@@ -2570,7 +2570,7 @@
       <c r="G7" s="15"/>
       <c r="H7" s="15"/>
     </row>
-    <row r="8" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A8" s="13"/>
       <c r="B8" s="19" t="s">
         <v>37</v>
@@ -2584,7 +2584,7 @@
       <c r="G8" s="15"/>
       <c r="H8" s="15"/>
     </row>
-    <row r="9" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A9" s="13"/>
       <c r="B9" s="19" t="s">
         <v>38</v>
@@ -2598,7 +2598,7 @@
       <c r="G9" s="15"/>
       <c r="H9" s="15"/>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A10" s="69"/>
       <c r="B10" s="69"/>
       <c r="C10" s="14"/>
@@ -2608,7 +2608,7 @@
       <c r="G10" s="25"/>
       <c r="H10" s="15"/>
     </row>
-    <row r="11" spans="1:18" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A11" s="69"/>
       <c r="B11" s="69"/>
       <c r="C11" s="14"/>
@@ -2618,7 +2618,7 @@
       <c r="G11" s="15"/>
       <c r="H11" s="15"/>
     </row>
-    <row r="12" spans="1:18" ht="18" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:18" ht="18" x14ac:dyDescent="0.4">
       <c r="A12" s="13"/>
       <c r="B12" s="28" t="s">
         <v>40</v>
@@ -2630,7 +2630,7 @@
       <c r="G12" s="15"/>
       <c r="H12" s="15"/>
     </row>
-    <row r="13" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="69"/>
       <c r="B13" s="69"/>
       <c r="C13" s="29"/>
@@ -2640,7 +2640,7 @@
       <c r="G13" s="15"/>
       <c r="H13" s="15"/>
     </row>
-    <row r="14" spans="1:18" ht="30" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:18" ht="28" x14ac:dyDescent="0.35">
       <c r="B14" s="45" t="s">
         <v>41</v>
       </c>
@@ -2684,7 +2684,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:18" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B15" s="32" t="s">
         <v>44</v>
       </c>
@@ -2728,7 +2728,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:18" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B16" s="34" t="s">
         <v>46</v>
       </c>
@@ -2775,7 +2775,7 @@
       <c r="Q16" s="15"/>
       <c r="R16" s="15"/>
     </row>
-    <row r="17" spans="2:15" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B17" s="34" t="s">
         <v>48</v>
       </c>
@@ -2819,7 +2819,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="2:15" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B18" s="34" t="s">
         <v>50</v>
       </c>
@@ -2863,7 +2863,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="2:15" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B19" s="34" t="s">
         <v>52</v>
       </c>
@@ -2907,7 +2907,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="2:15" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B20" s="34" t="s">
         <v>54</v>
       </c>
@@ -2951,7 +2951,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="2:15" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B21" s="34" t="s">
         <v>56</v>
       </c>
@@ -2995,7 +2995,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="2:15" ht="18" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:15" ht="18" x14ac:dyDescent="0.4">
       <c r="B22" s="67" t="s">
         <v>43</v>
       </c>
@@ -3037,7 +3037,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="24" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B24" s="66" t="s">
         <v>402</v>
       </c>
@@ -3055,7 +3055,7 @@
       <c r="N24" s="66"/>
       <c r="O24" s="66"/>
     </row>
-    <row r="25" spans="2:15" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
       <c r="D25" s="66"/>
@@ -3071,7 +3071,7 @@
       <c r="N25" s="66"/>
       <c r="O25" s="66"/>
     </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B26" s="66"/>
       <c r="C26" s="66"/>
       <c r="D26" s="66"/>
@@ -3087,7 +3087,7 @@
       <c r="N26" s="66"/>
       <c r="O26" s="66"/>
     </row>
-    <row r="27" spans="2:15" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B27" s="66"/>
       <c r="C27" s="66"/>
       <c r="D27" s="66"/>
@@ -3124,27 +3124,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54853DFE-3DA2-4431-9118-18B40B4CEBE8}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:S157"/>
-  <sheetFormatPr defaultColWidth="57.28515625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="57.26953125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="2.140625" style="4" customWidth="1"/>
-    <col min="2" max="2" width="14.42578125" style="4" customWidth="1"/>
-    <col min="3" max="3" width="27.7109375" style="4" customWidth="1"/>
-    <col min="4" max="4" width="69.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="33.5703125" style="16" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.42578125" style="16" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="82.5703125" style="16" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="19" width="18.42578125" style="4" customWidth="1"/>
-    <col min="20" max="16384" width="57.28515625" style="4"/>
+    <col min="1" max="1" width="2.1796875" style="4" customWidth="1"/>
+    <col min="2" max="2" width="14.453125" style="4" customWidth="1"/>
+    <col min="3" max="3" width="27.7265625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="69.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.54296875" style="16" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.453125" style="16" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="64.81640625" style="16" customWidth="1"/>
+    <col min="8" max="8" width="11.81640625" style="4" hidden="1" customWidth="1"/>
+    <col min="9" max="16" width="18.453125" style="4" hidden="1" customWidth="1"/>
+    <col min="17" max="17" width="18.453125" style="4" customWidth="1"/>
+    <col min="18" max="19" width="18.453125" style="4" hidden="1" customWidth="1"/>
+    <col min="20" max="16384" width="57.26953125" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="9" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:19" ht="9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="69"/>
       <c r="B1" s="69"/>
       <c r="C1" s="14"/>
       <c r="D1" s="14"/>
     </row>
-    <row r="2" spans="1:19" ht="18" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:19" ht="18" x14ac:dyDescent="0.35">
       <c r="A2" s="13"/>
       <c r="B2" s="17" t="s">
         <v>29</v>
@@ -3154,7 +3156,7 @@
       </c>
       <c r="D2" s="14"/>
     </row>
-    <row r="3" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A3" s="13"/>
       <c r="B3" s="17" t="s">
         <v>30</v>
@@ -3164,7 +3166,7 @@
       </c>
       <c r="D3" s="14"/>
     </row>
-    <row r="4" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A4" s="13"/>
       <c r="B4" s="19" t="s">
         <v>31</v>
@@ -3174,7 +3176,7 @@
       </c>
       <c r="D4" s="14"/>
     </row>
-    <row r="5" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A5" s="13"/>
       <c r="B5" s="19" t="s">
         <v>33</v>
@@ -3184,7 +3186,7 @@
       </c>
       <c r="D5" s="14"/>
     </row>
-    <row r="6" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A6" s="13"/>
       <c r="B6" s="19" t="s">
         <v>34</v>
@@ -3194,7 +3196,7 @@
       </c>
       <c r="D6" s="14"/>
     </row>
-    <row r="7" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A7" s="13"/>
       <c r="B7" s="19" t="s">
         <v>36</v>
@@ -3204,7 +3206,7 @@
       </c>
       <c r="D7" s="14"/>
     </row>
-    <row r="8" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A8" s="13"/>
       <c r="B8" s="19" t="s">
         <v>37</v>
@@ -3214,7 +3216,7 @@
       </c>
       <c r="D8" s="14"/>
     </row>
-    <row r="9" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A9" s="13"/>
       <c r="B9" s="19" t="s">
         <v>38</v>
@@ -3224,19 +3226,19 @@
       </c>
       <c r="D9" s="14"/>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A10" s="69"/>
       <c r="B10" s="69"/>
       <c r="C10" s="14"/>
       <c r="D10" s="14"/>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A11" s="69"/>
       <c r="B11" s="69"/>
       <c r="C11" s="14"/>
       <c r="D11" s="14"/>
     </row>
-    <row r="12" spans="1:19" ht="18" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:19" ht="18" x14ac:dyDescent="0.4">
       <c r="A12" s="13"/>
       <c r="B12" s="28" t="s">
         <v>58</v>
@@ -3244,14 +3246,14 @@
       <c r="C12" s="29"/>
       <c r="D12" s="30"/>
     </row>
-    <row r="13" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A13" s="69"/>
       <c r="B13" s="69"/>
       <c r="C13" s="29"/>
       <c r="D13" s="14"/>
       <c r="E13" s="15"/>
     </row>
-    <row r="14" spans="1:19" s="37" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:19" s="37" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="36"/>
       <c r="B14" s="43" t="s">
         <v>41</v>
@@ -3308,7 +3310,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A15" s="13"/>
       <c r="B15" s="38" t="s">
         <v>44</v>
@@ -3365,7 +3367,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A16" s="13"/>
       <c r="B16" s="38" t="s">
         <v>44</v>
@@ -3422,7 +3424,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A17" s="13"/>
       <c r="B17" s="38" t="s">
         <v>44</v>
@@ -3479,7 +3481,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A18" s="13"/>
       <c r="B18" s="38" t="s">
         <v>44</v>
@@ -3536,7 +3538,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A19" s="13"/>
       <c r="B19" s="38" t="s">
         <v>44</v>
@@ -3593,7 +3595,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A20" s="13"/>
       <c r="B20" s="38" t="s">
         <v>44</v>
@@ -3650,7 +3652,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A21" s="13"/>
       <c r="B21" s="38" t="s">
         <v>44</v>
@@ -3707,7 +3709,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A22" s="13"/>
       <c r="B22" s="38" t="s">
         <v>44</v>
@@ -3764,7 +3766,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A23" s="13"/>
       <c r="B23" s="38" t="s">
         <v>44</v>
@@ -3821,7 +3823,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A24" s="13"/>
       <c r="B24" s="38" t="s">
         <v>44</v>
@@ -3878,7 +3880,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A25" s="13"/>
       <c r="B25" s="38" t="s">
         <v>44</v>
@@ -3935,7 +3937,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A26" s="13"/>
       <c r="B26" s="38" t="s">
         <v>44</v>
@@ -3992,7 +3994,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A27" s="13"/>
       <c r="B27" s="38" t="s">
         <v>44</v>
@@ -4049,7 +4051,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A28" s="13"/>
       <c r="B28" s="38" t="s">
         <v>44</v>
@@ -4106,7 +4108,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A29" s="13"/>
       <c r="B29" s="38" t="s">
         <v>44</v>
@@ -4163,7 +4165,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A30" s="13"/>
       <c r="B30" s="38" t="s">
         <v>44</v>
@@ -4220,7 +4222,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A31" s="13"/>
       <c r="B31" s="38" t="s">
         <v>44</v>
@@ -4277,7 +4279,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A32" s="13"/>
       <c r="B32" s="38" t="s">
         <v>44</v>
@@ -4332,7 +4334,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A33" s="13"/>
       <c r="B33" s="38" t="s">
         <v>44</v>
@@ -4389,7 +4391,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A34" s="13"/>
       <c r="B34" s="38" t="s">
         <v>44</v>
@@ -4446,7 +4448,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A35" s="13"/>
       <c r="B35" s="38" t="s">
         <v>44</v>
@@ -4503,7 +4505,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A36" s="13"/>
       <c r="B36" s="38" t="s">
         <v>44</v>
@@ -4560,7 +4562,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A37" s="13"/>
       <c r="B37" s="38" t="s">
         <v>44</v>
@@ -4617,7 +4619,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A38" s="13"/>
       <c r="B38" s="38" t="s">
         <v>46</v>
@@ -4674,7 +4676,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="39" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A39" s="13"/>
       <c r="B39" s="38" t="s">
         <v>46</v>
@@ -4731,7 +4733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A40" s="13"/>
       <c r="B40" s="38" t="s">
         <v>46</v>
@@ -4788,7 +4790,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="41" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A41" s="13"/>
       <c r="B41" s="38" t="s">
         <v>46</v>
@@ -4845,7 +4847,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="42" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A42" s="13"/>
       <c r="B42" s="38" t="s">
         <v>46</v>
@@ -4902,7 +4904,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A43" s="13"/>
       <c r="B43" s="38" t="s">
         <v>46</v>
@@ -4959,7 +4961,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="44" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A44" s="13"/>
       <c r="B44" s="38" t="s">
         <v>46</v>
@@ -5016,7 +5018,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A45" s="13"/>
       <c r="B45" s="38" t="s">
         <v>46</v>
@@ -5073,7 +5075,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="46" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A46" s="13"/>
       <c r="B46" s="38" t="s">
         <v>46</v>
@@ -5130,7 +5132,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A47" s="13"/>
       <c r="B47" s="38" t="s">
         <v>46</v>
@@ -5187,7 +5189,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A48" s="13"/>
       <c r="B48" s="38" t="s">
         <v>46</v>
@@ -5244,7 +5246,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="49" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A49" s="13"/>
       <c r="B49" s="38" t="s">
         <v>46</v>
@@ -5301,7 +5303,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B50" s="38" t="s">
         <v>46</v>
       </c>
@@ -5357,7 +5359,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B51" s="38" t="s">
         <v>48</v>
       </c>
@@ -5413,7 +5415,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="52" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B52" s="38" t="s">
         <v>48</v>
       </c>
@@ -5469,7 +5471,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B53" s="38" t="s">
         <v>48</v>
       </c>
@@ -5525,7 +5527,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B54" s="38" t="s">
         <v>48</v>
       </c>
@@ -5581,7 +5583,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B55" s="38" t="s">
         <v>48</v>
       </c>
@@ -5637,7 +5639,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B56" s="38" t="s">
         <v>48</v>
       </c>
@@ -5693,7 +5695,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B57" s="38" t="s">
         <v>48</v>
       </c>
@@ -5749,7 +5751,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="58" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B58" s="38" t="s">
         <v>48</v>
       </c>
@@ -5805,7 +5807,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B59" s="38" t="s">
         <v>48</v>
       </c>
@@ -5861,7 +5863,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="60" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B60" s="38" t="s">
         <v>48</v>
       </c>
@@ -5917,7 +5919,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="61" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B61" s="38" t="s">
         <v>48</v>
       </c>
@@ -5973,7 +5975,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B62" s="38" t="s">
         <v>48</v>
       </c>
@@ -6029,7 +6031,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B63" s="38" t="s">
         <v>48</v>
       </c>
@@ -6085,7 +6087,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B64" s="38" t="s">
         <v>48</v>
       </c>
@@ -6141,7 +6143,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="65" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B65" s="38" t="s">
         <v>48</v>
       </c>
@@ -6197,7 +6199,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="66" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="66" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B66" s="38" t="s">
         <v>48</v>
       </c>
@@ -6253,7 +6255,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="67" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B67" s="38" t="s">
         <v>48</v>
       </c>
@@ -6309,7 +6311,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="68" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B68" s="38" t="s">
         <v>48</v>
       </c>
@@ -6365,7 +6367,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="69" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="69" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B69" s="38" t="s">
         <v>48</v>
       </c>
@@ -6419,7 +6421,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="70" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B70" s="38" t="s">
         <v>50</v>
       </c>
@@ -6475,7 +6477,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="71" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B71" s="38" t="s">
         <v>50</v>
       </c>
@@ -6531,7 +6533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="72" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B72" s="38" t="s">
         <v>50</v>
       </c>
@@ -6587,7 +6589,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="73" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="73" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B73" s="38" t="s">
         <v>50</v>
       </c>
@@ -6643,7 +6645,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="74" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="74" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B74" s="38" t="s">
         <v>50</v>
       </c>
@@ -6699,7 +6701,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="75" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="75" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B75" s="38" t="s">
         <v>50</v>
       </c>
@@ -6755,7 +6757,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="76" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B76" s="38" t="s">
         <v>50</v>
       </c>
@@ -6811,7 +6813,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="77" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="77" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B77" s="38" t="s">
         <v>50</v>
       </c>
@@ -6867,7 +6869,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="78" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B78" s="38" t="s">
         <v>50</v>
       </c>
@@ -6923,7 +6925,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="79" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="79" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B79" s="38" t="s">
         <v>50</v>
       </c>
@@ -6979,7 +6981,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="80" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B80" s="38" t="s">
         <v>50</v>
       </c>
@@ -7035,7 +7037,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="81" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B81" s="38" t="s">
         <v>50</v>
       </c>
@@ -7091,7 +7093,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="82" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="82" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B82" s="38" t="s">
         <v>50</v>
       </c>
@@ -7147,7 +7149,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="83" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B83" s="38" t="s">
         <v>50</v>
       </c>
@@ -7203,7 +7205,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="84" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B84" s="38" t="s">
         <v>50</v>
       </c>
@@ -7259,7 +7261,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="85" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B85" s="38" t="s">
         <v>50</v>
       </c>
@@ -7315,7 +7317,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="86" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B86" s="38" t="s">
         <v>50</v>
       </c>
@@ -7371,7 +7373,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="87" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B87" s="38" t="s">
         <v>50</v>
       </c>
@@ -7427,7 +7429,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="88" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B88" s="38" t="s">
         <v>50</v>
       </c>
@@ -7483,7 +7485,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="89" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="89" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B89" s="38" t="s">
         <v>50</v>
       </c>
@@ -7539,7 +7541,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="90" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B90" s="38" t="s">
         <v>50</v>
       </c>
@@ -7595,7 +7597,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="91" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B91" s="38" t="s">
         <v>50</v>
       </c>
@@ -7651,7 +7653,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="92" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B92" s="38" t="s">
         <v>50</v>
       </c>
@@ -7707,7 +7709,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="93" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B93" s="38" t="s">
         <v>52</v>
       </c>
@@ -7763,7 +7765,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="94" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B94" s="38" t="s">
         <v>52</v>
       </c>
@@ -7819,7 +7821,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="95" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B95" s="38" t="s">
         <v>52</v>
       </c>
@@ -7875,7 +7877,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="96" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="96" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B96" s="38" t="s">
         <v>52</v>
       </c>
@@ -7931,7 +7933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="97" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B97" s="38" t="s">
         <v>52</v>
       </c>
@@ -7987,7 +7989,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="98" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B98" s="38" t="s">
         <v>52</v>
       </c>
@@ -8043,7 +8045,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="99" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B99" s="38" t="s">
         <v>52</v>
       </c>
@@ -8099,7 +8101,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="100" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B100" s="38" t="s">
         <v>52</v>
       </c>
@@ -8155,7 +8157,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="101" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B101" s="38" t="s">
         <v>52</v>
       </c>
@@ -8211,7 +8213,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="102" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="102" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B102" s="38" t="s">
         <v>52</v>
       </c>
@@ -8267,7 +8269,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="103" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B103" s="38" t="s">
         <v>52</v>
       </c>
@@ -8323,7 +8325,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="104" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B104" s="38" t="s">
         <v>52</v>
       </c>
@@ -8379,7 +8381,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="105" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B105" s="38" t="s">
         <v>52</v>
       </c>
@@ -8435,7 +8437,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="106" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="106" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B106" s="38" t="s">
         <v>52</v>
       </c>
@@ -8491,7 +8493,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="107" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="107" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B107" s="38" t="s">
         <v>54</v>
       </c>
@@ -8547,7 +8549,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="108" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B108" s="38" t="s">
         <v>54</v>
       </c>
@@ -8603,7 +8605,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="109" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B109" s="38" t="s">
         <v>54</v>
       </c>
@@ -8659,7 +8661,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="110" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="110" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B110" s="38" t="s">
         <v>54</v>
       </c>
@@ -8715,7 +8717,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="111" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B111" s="38" t="s">
         <v>54</v>
       </c>
@@ -8771,7 +8773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="112" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B112" s="38" t="s">
         <v>54</v>
       </c>
@@ -8827,7 +8829,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="113" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="113" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B113" s="38" t="s">
         <v>54</v>
       </c>
@@ -8883,7 +8885,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="114" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B114" s="38" t="s">
         <v>54</v>
       </c>
@@ -8939,7 +8941,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="115" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B115" s="38" t="s">
         <v>54</v>
       </c>
@@ -8995,7 +8997,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="116" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B116" s="38" t="s">
         <v>54</v>
       </c>
@@ -9051,7 +9053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="117" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B117" s="38" t="s">
         <v>54</v>
       </c>
@@ -9107,7 +9109,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="118" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="118" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B118" s="38" t="s">
         <v>54</v>
       </c>
@@ -9163,7 +9165,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="119" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="119" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B119" s="38" t="s">
         <v>54</v>
       </c>
@@ -9219,7 +9221,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="120" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B120" s="38" t="s">
         <v>54</v>
       </c>
@@ -9275,7 +9277,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="121" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B121" s="38" t="s">
         <v>54</v>
       </c>
@@ -9331,7 +9333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="122" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B122" s="38" t="s">
         <v>54</v>
       </c>
@@ -9387,7 +9389,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="123" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B123" s="38" t="s">
         <v>54</v>
       </c>
@@ -9443,7 +9445,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="124" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B124" s="38" t="s">
         <v>54</v>
       </c>
@@ -9499,7 +9501,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="125" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B125" s="38" t="s">
         <v>54</v>
       </c>
@@ -9555,7 +9557,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="126" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B126" s="38" t="s">
         <v>54</v>
       </c>
@@ -9611,7 +9613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="127" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B127" s="38" t="s">
         <v>54</v>
       </c>
@@ -9667,7 +9669,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="128" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B128" s="38" t="s">
         <v>54</v>
       </c>
@@ -9723,7 +9725,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="129" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B129" s="38" t="s">
         <v>54</v>
       </c>
@@ -9779,7 +9781,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="130" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B130" s="38" t="s">
         <v>54</v>
       </c>
@@ -9835,7 +9837,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="131" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="131" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B131" s="38" t="s">
         <v>56</v>
       </c>
@@ -9891,7 +9893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="132" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B132" s="38" t="s">
         <v>56</v>
       </c>
@@ -9947,7 +9949,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="133" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="133" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B133" s="38" t="s">
         <v>56</v>
       </c>
@@ -10003,7 +10005,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="134" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B134" s="38" t="s">
         <v>56</v>
       </c>
@@ -10059,7 +10061,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="135" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="135" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B135" s="38" t="s">
         <v>56</v>
       </c>
@@ -10115,7 +10117,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="136" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B136" s="38" t="s">
         <v>56</v>
       </c>
@@ -10171,7 +10173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="137" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B137" s="38" t="s">
         <v>56</v>
       </c>
@@ -10227,7 +10229,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="138" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B138" s="38" t="s">
         <v>56</v>
       </c>
@@ -10283,7 +10285,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="139" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B139" s="38" t="s">
         <v>56</v>
       </c>
@@ -10339,7 +10341,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="140" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B140" s="38" t="s">
         <v>56</v>
       </c>
@@ -10395,7 +10397,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="141" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="141" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B141" s="38" t="s">
         <v>56</v>
       </c>
@@ -10451,7 +10453,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="142" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="142" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B142" s="38" t="s">
         <v>56</v>
       </c>
@@ -10507,7 +10509,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="143" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B143" s="38" t="s">
         <v>56</v>
       </c>
@@ -10563,7 +10565,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="144" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B144" s="38" t="s">
         <v>56</v>
       </c>
@@ -10619,7 +10621,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="145" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B145" s="38" t="s">
         <v>56</v>
       </c>
@@ -10675,7 +10677,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="146" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="146" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B146" s="38" t="s">
         <v>56</v>
       </c>
@@ -10731,7 +10733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="147" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B147" s="38" t="s">
         <v>56</v>
       </c>
@@ -10787,7 +10789,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="148" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B148" s="38" t="s">
         <v>56</v>
       </c>
@@ -10843,7 +10845,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="149" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B149" s="38" t="s">
         <v>56</v>
       </c>
@@ -10899,7 +10901,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="150" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="150" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B150" s="38" t="s">
         <v>56</v>
       </c>
@@ -10955,7 +10957,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="151" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B151" s="38" t="s">
         <v>56</v>
       </c>
@@ -11011,7 +11013,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="152" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B152" s="32" t="s">
         <v>56</v>
       </c>
@@ -11067,7 +11069,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="154" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B154" s="70" t="s">
         <v>402</v>
       </c>
@@ -11077,7 +11079,7 @@
       <c r="F154" s="70"/>
       <c r="G154" s="70"/>
     </row>
-    <row r="155" spans="2:19" x14ac:dyDescent="0.2">
+    <row r="155" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B155" s="70"/>
       <c r="C155" s="70"/>
       <c r="D155" s="70"/>
@@ -11085,7 +11087,7 @@
       <c r="F155" s="70"/>
       <c r="G155" s="70"/>
     </row>
-    <row r="156" spans="2:19" x14ac:dyDescent="0.2">
+    <row r="156" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B156" s="70"/>
       <c r="C156" s="70"/>
       <c r="D156" s="70"/>
@@ -11093,7 +11095,7 @@
       <c r="F156" s="70"/>
       <c r="G156" s="70"/>
     </row>
-    <row r="157" spans="2:19" x14ac:dyDescent="0.2">
+    <row r="157" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B157" s="47"/>
       <c r="C157" s="47"/>
       <c r="D157" s="47"/>
@@ -11346,15 +11348,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
@@ -11364,6 +11357,15 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11387,14 +11389,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F436471D-C45C-4DAE-8C21-752C3CF7A405}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7706BC6D-3A42-4EE7-8F02-E43240B61A4E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
@@ -11412,6 +11406,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F436471D-C45C-4DAE-8C21-752C3CF7A405}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{37c354b2-85b0-47f5-b222-07b48d774ee3}" enabled="0" method="" siteId="{37c354b2-85b0-47f5-b222-07b48d774ee3}" removed="1"/>

</xml_diff>